<commit_message>
chore: .env.example에 SUPER_ADMIN_JWT_SECRET 항목 추가 및 청연컨설팅 사용자 템플릿 갱신
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGypjKDKYkSvEtuDtrUMHg
</commit_message>
<xml_diff>
--- a/templates/chungyeon-consulting-users-template.xlsx
+++ b/templates/chungyeon-consulting-users-template.xlsx
@@ -1,19 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10628"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A556F835-15A2-D34F-8C08-02C2022ED761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="660" windowWidth="51200" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="사용자목록" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="_lists" state="veryHidden" r:id="rId5"/>
-    <sheet sheetId="3" name="작성안내" state="visible" r:id="rId6"/>
+    <sheet name="사용자목록" sheetId="1" r:id="rId1"/>
+    <sheet name="_lists" sheetId="2" state="veryHidden" r:id="rId2"/>
+    <sheet name="작성안내" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">사용자목록!$A$1:$E$46</definedName>
+  </definedNames>
+  <calcPr calcId="171027" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="53">
   <si>
     <t>userid (아이디)</t>
   </si>
@@ -151,22 +158,61 @@
   </si>
   <si>
     <t>경영지원본부 &gt; 경영지원팀  |  경영지원본부 &gt; 재무팀  |  경영지원본부 &gt; 인사팀  |  경영지원본부 &gt; 총무팀  |  환경사업본부 &gt; 환경측정팀  |  환경사업본부 &gt; 수질관리팀  |  환경사업본부 &gt; 대기관리팀  |  환경사업본부 &gt; 실험분석팀  |  컨설팅본부 &gt; 환경컨설팅팀  |  컨설팅본부 &gt; 안전컨설팅팀  |  컨설팅본부 &gt; 기술지원팀  |  영업본부 &gt; 영업1팀  |  영업본부 &gt; 영업2팀  |  영업본부 &gt; 고객지원팀</t>
+  </si>
+  <si>
+    <t>신창국</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>정혜종</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>김흥래</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>김석현</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>팀장</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>기술연구팀</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>오관균</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -200,7 +246,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -536,9 +582,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E45"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E47"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -547,7 +593,7 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,12 +610,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -581,12 +627,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -598,12 +644,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -615,7 +661,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -632,7 +678,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -649,12 +695,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -666,7 +712,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -683,7 +729,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -700,7 +746,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -717,7 +763,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -734,7 +780,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -751,12 +797,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
         <v>10</v>
@@ -768,7 +814,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -785,7 +831,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -802,7 +848,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -819,7 +865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -836,7 +882,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -853,7 +899,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -870,7 +916,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -887,7 +933,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -904,7 +950,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>5</v>
       </c>
@@ -921,7 +967,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>5</v>
       </c>
@@ -938,7 +984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>5</v>
       </c>
@@ -955,7 +1001,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
         <v>5</v>
       </c>
@@ -972,7 +1018,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -989,7 +1035,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
         <v>5</v>
       </c>
@@ -1006,7 +1052,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>5</v>
       </c>
@@ -1023,7 +1069,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
         <v>5</v>
       </c>
@@ -1040,7 +1086,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
         <v>5</v>
       </c>
@@ -1057,7 +1103,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
         <v>5</v>
       </c>
@@ -1074,7 +1120,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -1091,7 +1137,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
         <v>5</v>
       </c>
@@ -1108,12 +1154,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="C34" t="s">
         <v>10</v>
@@ -1125,10 +1171,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>5</v>
-      </c>
+    <row r="35" spans="1:5">
       <c r="B35" t="s">
         <v>5</v>
       </c>
@@ -1142,7 +1185,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -1159,12 +1202,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="C37" t="s">
         <v>10</v>
@@ -1176,7 +1219,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -1193,7 +1236,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
         <v>5</v>
       </c>
@@ -1210,7 +1253,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5">
       <c r="A40" t="s">
         <v>5</v>
       </c>
@@ -1227,7 +1270,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5">
       <c r="A41" t="s">
         <v>5</v>
       </c>
@@ -1244,7 +1287,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5">
       <c r="A42" t="s">
         <v>5</v>
       </c>
@@ -1261,12 +1304,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="C43" t="s">
         <v>10</v>
@@ -1278,7 +1321,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5">
       <c r="A44" t="s">
         <v>5</v>
       </c>
@@ -1295,7 +1338,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5">
       <c r="A45" t="s">
         <v>5</v>
       </c>
@@ -1312,123 +1355,160 @@
         <v>8</v>
       </c>
     </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" t="s">
+        <v>50</v>
+      </c>
+      <c r="D46" t="s">
+        <v>51</v>
+      </c>
+      <c r="E46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" t="s">
+        <v>51</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="역할 오류" error="허용 역할: 재정팀장, 회계, 팀장, 사용자" sqref="C10:C45">
+  <autoFilter ref="A1:E46" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="역할 오류" error="허용 역할: 재정팀장, 회계, 팀장, 사용자" sqref="C2:C45 C47" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"재정팀장,회계,팀장,사용자"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="역할 오류" error="허용 역할: 재정팀장, 회계, 팀장, 사용자" sqref="C2:C45">
-      <formula1>"재정팀장,회계,팀장,사용자"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D10:D45">
-      <formula1>_lists!$A$1:$A$14</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D45">
-      <formula1>_lists!$A$1:$A$14</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E10:E45">
-      <formula1>"Y,N"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E2:E45">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E47" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
+          <x14:formula1>
+            <xm:f>_lists!$A$1:$A$14</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D45</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A14"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1">
       <c r="A8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1">
       <c r="A10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1">
       <c r="A11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1">
       <c r="A12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1">
       <c r="A13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1">
       <c r="A14" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="2" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>25</v>
       </c>
@@ -1436,7 +1516,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1444,7 +1524,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1452,7 +1532,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1460,7 +1540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1468,7 +1548,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1476,7 +1556,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1484,7 +1564,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1492,7 +1572,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1500,7 +1580,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -1508,7 +1588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>36</v>
       </c>
@@ -1516,7 +1596,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1524,7 +1604,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1532,7 +1612,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>42</v>
       </c>
@@ -1540,7 +1620,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1548,7 +1628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -1557,7 +1637,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>